<commit_message>
feat: implement template management API and visual game builder component
</commit_message>
<xml_diff>
--- a/Тестова ситуація.xlsx
+++ b/Тестова ситуація.xlsx
@@ -3,7 +3,8 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
   <workbookPr/>
   <sheets>
-    <sheet state="visible" name="Аркуш1" sheetId="1" r:id="rId5"/>
+    <sheet state="visible" name="Ситуація" sheetId="1" r:id="rId5"/>
+    <sheet state="visible" name="Результати" sheetId="2" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr/>
@@ -11,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="55" uniqueCount="55">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="79" uniqueCount="79">
   <si>
     <t>СИТУАЦІЯ: До розважального центру завітала гостя з дитиною (на вигляд трохи більше року). 
 Мама сіла за стіл з дитиною. Ваші дії:</t>
@@ -129,10 +130,52 @@
         <rFont val="Arial"/>
         <color theme="1"/>
       </rPr>
-      <t>:
-ААА - 100% WOW-сервіс. Ти швидко реагуєш та підходиш до гостей. Ти не забуваєш про дитяче крісло та інші дрібниці, які впливають на якісний сервіс. Твої дії спрямовані на комфорт гостя та формують довіру до закладу.
-ААВ - 100% WOW-сервіс. Ти швидко реагуєш та підходиш до гостей. Ти не забуваєш про дитяче крісло та інші дрібниці, які впливають на якісний сервіс. Твої дії спрямовані на комфорт гостя та формують довіру до закладу.
-ААС - 100% WOW-сервіс. Ти швидко реагуєш та підходиш до гостей. Ти не забуваєш про дитяче крісло та інші дрібниці, які впливають на якісний сервіс. Твої дії створюють відчуття турботи та зміцнюють прихильність гості до закладу.
+      <t xml:space="preserve">:
+ААА - 100%  </t>
+    </r>
+    <r>
+      <rPr>
+        <rFont val="Arial"/>
+        <color rgb="FF38761D"/>
+      </rPr>
+      <t>Ти швидко реагуєш та підходиш до гостей. Ти не забуваєш про дитяче крісло та інші дрібниці, які впливають на якісний сервіс. Твої дії спрямовані на комфорт гостя та формують довіру до закладу.</t>
+    </r>
+    <r>
+      <rPr>
+        <rFont val="Arial"/>
+        <color theme="1"/>
+      </rPr>
+      <t xml:space="preserve">
+ААВ - 100%  </t>
+    </r>
+    <r>
+      <rPr>
+        <rFont val="Arial"/>
+        <color rgb="FF38761D"/>
+      </rPr>
+      <t>Ти швидко реагуєш та підходиш до гостей. Ти не забуваєш про дитяче крісло та інші дрібниці, які впливають на якісний сервіс. Твої дії спрямовані на комфорт гостя та формують довіру до закладу.</t>
+    </r>
+    <r>
+      <rPr>
+        <rFont val="Arial"/>
+        <color theme="1"/>
+      </rPr>
+      <t xml:space="preserve">
+ААС - 100%  </t>
+    </r>
+    <r>
+      <rPr>
+        <rFont val="Arial"/>
+        <color rgb="FF38761D"/>
+      </rPr>
+      <t>Ти швидко реагуєш та підходиш до гостей. Ти не забуваєш про дитяче крісло та інші дрібниці, які впливають на якісний сервіс. Твої дії створюють відчуття турботи та зміцнюють прихильність гості до закладу.</t>
+    </r>
+    <r>
+      <rPr>
+        <rFont val="Arial"/>
+        <color theme="1"/>
+      </rPr>
+      <t xml:space="preserve">
 ААD - 70%. Ти дієш правильно, але не завжди достатньо. Принести стілець для дитини - це дуже добре, але не забувай про подальше обслуговування, поки гостя обирає страви, запропонуй чай або каву. Трішки зусиль і ти перетвориш звичайний сервіс на WOW-рівень.</t>
     </r>
   </si>
@@ -453,8 +496,22 @@
         <rFont val="Arial"/>
         <color theme="1"/>
       </rPr>
-      <t>:
-АDА - 100% WOW-сервіс. Ти швидко реагуєш та підходиш до гостей. Ти не забуваєш про дитяче крісло та інші дрібниці, які впливають на якісний сервіс. Твої дії створюють відчуття турботи та зміцнюють прихильність гості до закладу.
+      <t xml:space="preserve">:
+АDА - 100%  </t>
+    </r>
+    <r>
+      <rPr>
+        <rFont val="Arial"/>
+        <color rgb="FF38761D"/>
+      </rPr>
+      <t>Ти швидко реагуєш та підходиш до гостей. Ти не забуваєш про дитяче крісло та інші дрібниці, які впливають на якісний сервіс. Твої дії створюють відчуття турботи та зміцнюють прихильність гості до закладу.</t>
+    </r>
+    <r>
+      <rPr>
+        <rFont val="Arial"/>
+        <color theme="1"/>
+      </rPr>
+      <t xml:space="preserve">
 АDВ - 70%. Ти дієш правильно, але не завжди достатньо. Принести стілець для дитини - це дуже добре, але не забувай про подальше обслуговування, поки гостя обирає страви, запропонуй чай або каву. Трішки зусиль і ти перетвориш звичайний сервіс на WOW-рівень.
 АDС - 70%. Ти дієш правильно, але не завжди достатньо. Принести стілець для дитини - це дуже добре, але не забувай про подальше обслуговування, поки гостя обирає страви, запропонуй чай або каву. Трішки зусиль і ти перетвориш звичайний сервіс на WOW-рівень.
 АDD - 93% Ти впевнено та своєчасно реагуєш на ситуацію. Помічаєш важливі деталі та створюєш для гостя відчуття турботи й професіоналізму. Не забувай розгортати меню перед гостями - це важливий прояв турботи та сервісної культури.</t>
@@ -580,10 +637,52 @@
         <rFont val="Arial"/>
         <color theme="1"/>
       </rPr>
-      <t>:
-BАА - 100% WOW-сервіс. Ти швидко реагуєш та підходиш до гостей. Ти не забуваєш про дитяче крісло та інші дрібниці, які впливають на якісний сервіс. Твої дії створюють відчуття турботи та зміцнюють прихильність гості до закладу.
-BАВ - 100% WOW-сервіс. Ти швидко реагуєш та підходиш до гостей. Ти не забуваєш про дитяче крісло та інші дрібниці, які впливають на якісний сервіс. Твої дії створюють відчуття турботи та зміцнюють прихильність гості до закладу.
-BАС - 100% WOW-сервіс. Ти швидко реагуєш та підходиш до гостей. Ти не забуваєш про дитяче крісло та інші дрібниці, які впливають на якісний сервіс. Твої дії створюють відчуття турботи та зміцнюють прихильність гості до закладу.
+      <t xml:space="preserve">:
+BАА - 100%  </t>
+    </r>
+    <r>
+      <rPr>
+        <rFont val="Arial"/>
+        <color rgb="FF38761D"/>
+      </rPr>
+      <t>Ти швидко реагуєш та підходиш до гостей. Ти не забуваєш про дитяче крісло та інші дрібниці, які впливають на якісний сервіс. Твої дії створюють відчуття турботи та зміцнюють прихильність гості до закладу.</t>
+    </r>
+    <r>
+      <rPr>
+        <rFont val="Arial"/>
+        <color theme="1"/>
+      </rPr>
+      <t xml:space="preserve">
+BАВ - 100% </t>
+    </r>
+    <r>
+      <rPr>
+        <rFont val="Arial"/>
+        <color rgb="FF38761D"/>
+      </rPr>
+      <t>Ти швидко реагуєш та підходиш до гостей. Ти не забуваєш про дитяче крісло та інші дрібниці, які впливають на якісний сервіс. Твої дії створюють відчуття турботи та зміцнюють прихильність гості до закладу.</t>
+    </r>
+    <r>
+      <rPr>
+        <rFont val="Arial"/>
+        <color theme="1"/>
+      </rPr>
+      <t xml:space="preserve">
+BАС - 100%  </t>
+    </r>
+    <r>
+      <rPr>
+        <rFont val="Arial"/>
+        <color rgb="FF38761D"/>
+      </rPr>
+      <t>Ти швидко реагуєш та підходиш до гостей. Ти не забуваєш про дитяче крісло та інші дрібниці, які впливають на якісний сервіс. Твої дії створюють відчуття турботи та зміцнюють прихильність гості до закладу.</t>
+    </r>
+    <r>
+      <rPr>
+        <rFont val="Arial"/>
+        <color theme="1"/>
+      </rPr>
+      <t xml:space="preserve">
 BАD - 70%. Ти дієш правильно, але не завжди достатньо. Принести стілець для дитини - це дуже добре, але не забувай про подальше обслуговування, поки гостя обирає страви, запропонуй чай або каву. Трішки зусиль і ти перетвориш звичайний сервіс на WOW-рівень.</t>
     </r>
   </si>
@@ -897,11 +996,32 @@
         <rFont val="Arial"/>
         <color theme="1"/>
       </rPr>
-      <t>:
-BDА - 100% WOW-сервіс. Ти швидко реагуєш та підходиш до гостей. Ти не забуваєш про дитяче крісло та інші дрібниці, які впливають на якісний сервіс. Твої дії створюють відчуття турботи та зміцнюють прихильність гості до закладу.
+      <t xml:space="preserve">:
+BDА - 100% </t>
+    </r>
+    <r>
+      <rPr>
+        <rFont val="Arial"/>
+        <color rgb="FF38761D"/>
+      </rPr>
+      <t>Ти швидко реагуєш та підходиш до гостей. Ти не забуваєш про дитяче крісло та інші дрібниці, які впливають на якісний сервіс. Твої дії створюють відчуття турботи та зміцнюють прихильність гості до закладу.</t>
+    </r>
+    <r>
+      <rPr>
+        <rFont val="Arial"/>
+        <color theme="1"/>
+      </rPr>
+      <t xml:space="preserve">
 BDВ - 70% Ти дієш правильно, але не завжди достатньо. Принести стілець для дитини - це дуже добре, але не забувай про подальше обслуговування, поки гостя обирає страви, запропонуй чай або каву. Трішки зусиль і ти перетвориш звичайний сервіс на WOW-рівень.
 BDС - 70% Ти дієш правильно, але не завжди достатньо. Принести стілець для дитини - це дуже добре, але не забувай про подальше обслуговування, поки гостя обирає страви, запропонуй чай або каву. Трішки зусиль і ти перетвориш звичайний сервіс на WOW-рівень.
-BDD - 96% WOW-сервіс. Ти швидко реагуєш та підходиш до гостей. Ти не забуваєш про дитяче крісло та інші дрібниці, які впливають на якісний сервіс. Не забувай розгортати меню перед гостями - це важливий прояв турботи та сервісної культури.Твої дії створюють відчуття турботи та зміцнюють прихильність гості до закладу.</t>
+BDD - 96% </t>
+    </r>
+    <r>
+      <rPr>
+        <rFont val="Arial"/>
+        <color rgb="FF38761D"/>
+      </rPr>
+      <t>Ти швидко реагуєш та підходиш до гостей. Ти не забуваєш про дитяче крісло та інші дрібниці, які впливають на якісний сервіс. Не забувай розгортати меню перед гостями - це важливий прояв турботи та сервісної культури.Твої дії створюють відчуття турботи та зміцнюють прихильність гості до закладу.</t>
     </r>
   </si>
   <si>
@@ -1022,10 +1142,39 @@
         <color theme="1"/>
       </rPr>
       <t xml:space="preserve">:
-CАА - 100% WOW-сервіс. Ти швидко реагуєш та підходиш до гостей. Ти не забуваєш про дитяче крісло та інші дрібниці, які впливають на якісний сервіс. Твої дії створюють відчуття турботи та зміцнюють прихильність гості до закладу.
+CАА - 100% </t>
+    </r>
+    <r>
+      <rPr>
+        <rFont val="Arial"/>
+        <color rgb="FF38761D"/>
+      </rPr>
+      <t xml:space="preserve">Ти швидко реагуєш та підходиш до гостей. Ти не забуваєш про дитяче крісло та інші дрібниці, які впливають на якісний сервіс. Твої дії створюють відчуття турботи та зміцнюють прихильність гості до закладу.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <rFont val="Arial"/>
+        <color theme="1"/>
+      </rPr>
+      <t xml:space="preserve">
 CАВ - 73% Ти загалом правильно вів ситуацію, однак остання дія суттєво знизила твій рівень сервісу. Поставити меню на стіл і повідомити гостю, що ти не її офіціант і зараз до неї підійде її офіціант — це формальний підхід. Гостя залишилася без супроводу та відчуття турботи. Навіть якщо це не твій стіл, важливо прийняти замовлення самостійно, а потім передати його колезі. 
 CАС - 70% Ти загалом правильно вів ситуацію, однак остання дія суттєво знизила твій рівень сервісу. Поставити меню на стіл і повідомити гостю, що ти не її офіціант, запропонувавши скористатися QR-кодом — це формальний підхід. Гостя залишилася без супроводу та відчуття турботи. Навіть якщо це не твій стіл, важливо прийняти замовлення самостійно, а потім передати його колезі. 
-CАD - 100% WOW-сервіс. Ти швидко реагуєш та підходиш до гостей. Ти не забуваєш про дитяче крісло та інші дрібниці, які впливають на якісний сервіс. Твої дії створюють відчуття турботи та зміцнюють прихильність гості до закладу.
+CАD - 100%  </t>
+    </r>
+    <r>
+      <rPr>
+        <rFont val="Arial"/>
+        <color rgb="FF38761D"/>
+      </rPr>
+      <t>Ти швидко реагуєш та підходиш до гостей. Ти не забуваєш про дитяче крісло та інші дрібниці, які впливають на якісний сервіс. Твої дії створюють відчуття турботи та зміцнюють прихильність гості до закладу.</t>
+    </r>
+    <r>
+      <rPr>
+        <rFont val="Arial"/>
+        <color theme="1"/>
+      </rPr>
+      <t xml:space="preserve">
 </t>
     </r>
   </si>
@@ -1129,7 +1278,21 @@
 CВА - 63% Ти правильно залучив колегу до обслуговування його столу — це командна взаємодія.
 Проте повторне нагадування замість особистого втручання уповільнило вирішення ситуації. У подібних ситуаціях найсильніша позиція — взяти відповідальність і забезпечити сервіс тут і зараз, а внутрішні питання вирішувати після зміни.
 CВВ - 86% Ти дієш у межах командної взаємодії та контролюєш ситуацію — це правильно.
-Ти не ігноруєш проблему і намагаєшся залучити відповідального офіціанта. Проте нагадування, навіть особисте, не завжди дорівнює вирішенню ситуації. Поки триває комунікація між колегами, гість продовжує чекати. У таких випадках найсильніше рішення — або прийняти замовлення самостійно
+Ти не ігноруєш проблему і намагаєшся залучити відповідального офіціанта. Проте нагадування, навіть особисте, не завжди дорівнює вирішенню ситуації. Поки триває комунікація між колегами, гість продовжує чекати. У таких випадках найсильніше рішення —</t>
+    </r>
+    <r>
+      <rPr>
+        <rFont val="Arial"/>
+        <color rgb="FF38761D"/>
+      </rPr>
+      <t xml:space="preserve"> це </t>
+    </r>
+    <r>
+      <rPr>
+        <rFont val="Arial"/>
+        <color theme="1"/>
+      </rPr>
+      <t>прийняти замовлення самостійно.
 CВС - 93% Ти дієш як частина команди та не залишаєш ситуацію без контролю.
 Залучити колегу та запропонувати допомогу особисто - це правильне рішення. Важливо швидко реагувати та не допускати довгого очікування гостем офіціанта.
 CВD - 60% Публічна критика колеги в залі, при гостях та команді, демонструє непрофесійність і відсутність сервісної культури. Робочі моменти не вирішуються при гостях. У подібних ситуаціях найсильніша позиція — взяти відповідальність і забезпечити сервіс тут і зараз, а внутрішні питання вирішувати після зміни.</t>
@@ -1774,6 +1937,85 @@
 DDС - 0% Твої дії абсолютно не відповідають стандартам сервісу. Ігнорування ситуації та позиція «я не відповідаю за чужі столи» демонструють повну відсутність командного мислення. Гість не повинен бачити поділ на «мій» і «чужий» стіл. Для нього є один заклад і одна команда.
 DDD - 0% Твої дії абсолютно не відповідають стандартам сервісу. Твоя позиція демонструє повне перекладання відповідальності та відсутність командного підходу. Фраза «я не буду слідкувати за чужими столами» суперечить стандартам сервісу. Для гостя немає «чужих» офіціантів — є заклад як єдина команда. Навіть при високому навантаженні важливо не відмежовуватись від проблеми, а знайти рішення або передати її так, щоб гість не залишився без уваги.</t>
     </r>
+  </si>
+  <si>
+    <t>Результат</t>
+  </si>
+  <si>
+    <t>Оцінка</t>
+  </si>
+  <si>
+    <t>коментар</t>
+  </si>
+  <si>
+    <t>95-100%</t>
+  </si>
+  <si>
+    <t>WOW-СЕРВІС</t>
+  </si>
+  <si>
+    <t>WOW-сервіс. Ти швидко реагуєш та підходиш до гостей. Ти не забуваєш про дитяче крісло та інші дрібниці, які впливають на якісний сервіс. Твої дії спрямовані на комфорт гостя та формують довіру до закладу.</t>
+  </si>
+  <si>
+    <t>94-90%</t>
+  </si>
+  <si>
+    <t>ВІДМІННИЙ РІВЕНЬ</t>
+  </si>
+  <si>
+    <t>Ти обираєш вірний напрямок, але не використовуєш усі можливості сервісу. Гість отримує гарне обслуговування та увагу. Ти дуже близько до стабільного WOW-рівня.</t>
+  </si>
+  <si>
+    <t>89-80%</t>
+  </si>
+  <si>
+    <t>ХОРОШИЙ РІВЕНЬ</t>
+  </si>
+  <si>
+    <t>Ти дієш у межах командної взаємодії та контролюєш ситуацію — це правильно.
+Ти не ігноруєш проблему і намагаєшся залучити відповідального офіціанта. Проте нагадування, навіть особисте, не завжди дорівнює вирішенню ситуації. Поки триває комунікація між колегами, гість продовжує чекати. У таких випадках найсильніше рішення — або прийняти замовлення самостійно</t>
+  </si>
+  <si>
+    <t>79-70%</t>
+  </si>
+  <si>
+    <t>ПОТРІБНЕ ПОКРАЩЕННЯ</t>
+  </si>
+  <si>
+    <t>Ти дієш правильно, але не завжди достатньо. Трішки зусиль і ти перетвориш звичайний сервіс на WOW-рівень.</t>
+  </si>
+  <si>
+    <t>69-50%</t>
+  </si>
+  <si>
+    <t>ПОТРІБНА ОСОБЛИВА УВАГА</t>
+  </si>
+  <si>
+    <t>Гість не отримує гарного обслуговування, не відчуває турботу. У тебе бракує проактивності та уваги до деталей: допомоги з комфортом дитини, додаткових пропозицій. Зосередься на відповідальності та ініціативності — саме вони піднімають сервіс на вищий рівень. 
+Публічна критика колеги в залі, при гостях та команді, демонструє непрофесійність і відсутність сервісної культури. Робочі моменти не вирішуються при гостях. 
+Для гостя не існує «чужих» офіціантів — є заклад як єдина команда. Такий підхід демонструє відсутність включеності, ініціативи та відповідальності.
+ Помилка можлива. Важливо — як швидко ти її виправляєш.</t>
+  </si>
+  <si>
+    <t>49-30%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">КРИТИЧНИЙ РІВЕНЬ </t>
+  </si>
+  <si>
+    <t>подальша пасивність значно знизила якість сервісу. Ігнорування ситуації та фраза «це не моя зона відповідальності» демонструють байдужість до гостя та відсутність командного мислення. Для гостя не існує поділу на «мій» і «чужий» стіл — є заклад, який повинен забезпечити сервіс.Такий підхід створює ризик конфлікту, негативного відгуку та втрати лояльності.
+подальша позиція повністю суперечить стандартам сервісу. Ігнорування ситуації та фраза «це відповідальність старшого офіціанта» демонструють відмову від командної роботи та відповідальності за гостя. Навіть при великому навантаженні гість не повинен залишатися без уваги. Внутрішні ролі не можуть бути виправданням для бездіяльності.</t>
+  </si>
+  <si>
+    <t>29-0%</t>
+  </si>
+  <si>
+    <t>ПРОВАЛ</t>
+  </si>
+  <si>
+    <t>Твої дії абсолютно не відповідають рівню сервісу. Публічна критика колеги в залі, при гостях та команді, демонструє непрофесійність і відсутність сервісної культури. Робочі моменти не вирішуються при гостях. У подібних ситуаціях найсильніша позиція — взяти відповідальність і забезпечити сервіс тут і зараз, а внутрішні питання вирішувати після зміни.
+Гість не повинен відчувати внутрішні труднощі команди — він очікує увагу та сервіс.
+Твоя позиція демонструє повне перекладання відповідальності та відсутність командного підходу. Фраза «я не буду слідкувати за чужими столами» суперечить стандартам сервісу. Для гостя немає «чужих» офіціантів — є заклад як єдина команда. Навіть при високому навантаженні важливо не відмежовуватись від проблеми, а знайти рішення або передати її так, щоб гість не залишився без уваги.</t>
   </si>
 </sst>
 </file>
@@ -1807,12 +2049,54 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="9">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="lightGray"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF6AA84F"/>
+        <bgColor rgb="FF6AA84F"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFB6D7A8"/>
+        <bgColor rgb="FFB6D7A8"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFD9EAD3"/>
+        <bgColor rgb="FFD9EAD3"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFD966"/>
+        <bgColor rgb="FFFFD966"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF4CCCC"/>
+        <bgColor rgb="FFF4CCCC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFEA9999"/>
+        <bgColor rgb="FFEA9999"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFE06666"/>
+        <bgColor rgb="FFE06666"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="5">
@@ -1865,7 +2149,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="18">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -1890,6 +2174,30 @@
     <xf borderId="2" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
+    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment shrinkToFit="0" wrapText="1"/>
+    </xf>
+    <xf borderId="2" fillId="2" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment readingOrder="0"/>
+    </xf>
+    <xf borderId="2" fillId="3" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment readingOrder="0"/>
+    </xf>
+    <xf borderId="2" fillId="4" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment readingOrder="0"/>
+    </xf>
+    <xf borderId="2" fillId="5" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment readingOrder="0"/>
+    </xf>
+    <xf borderId="2" fillId="6" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment readingOrder="0"/>
+    </xf>
+    <xf borderId="2" fillId="7" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment readingOrder="0"/>
+    </xf>
+    <xf borderId="2" fillId="8" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment readingOrder="0"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle xfId="0" name="Normal" builtinId="0"/>
@@ -1899,6 +2207,10 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
+</file>
+
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
 </file>
 
@@ -2343,4 +2655,3085 @@
   </mergeCells>
   <drawing r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="0" summaryRight="0"/>
+  </sheetPr>
+  <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
+  <cols>
+    <col customWidth="1" min="1" max="1" width="16.75"/>
+    <col customWidth="1" min="2" max="2" width="31.88"/>
+    <col customWidth="1" min="3" max="3" width="98.13"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="C1" s="10"/>
+    </row>
+    <row r="2">
+      <c r="C2" s="10"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="C3" s="4" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="B4" s="11" t="s">
+        <v>59</v>
+      </c>
+      <c r="C4" s="4" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="s">
+        <v>61</v>
+      </c>
+      <c r="B5" s="12" t="s">
+        <v>62</v>
+      </c>
+      <c r="C5" s="4" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="s">
+        <v>64</v>
+      </c>
+      <c r="B6" s="13" t="s">
+        <v>65</v>
+      </c>
+      <c r="C6" s="4" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="s">
+        <v>67</v>
+      </c>
+      <c r="B7" s="14" t="s">
+        <v>68</v>
+      </c>
+      <c r="C7" s="4" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="s">
+        <v>70</v>
+      </c>
+      <c r="B8" s="15" t="s">
+        <v>71</v>
+      </c>
+      <c r="C8" s="4" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="s">
+        <v>73</v>
+      </c>
+      <c r="B9" s="16" t="s">
+        <v>74</v>
+      </c>
+      <c r="C9" s="4" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="s">
+        <v>76</v>
+      </c>
+      <c r="B10" s="17" t="s">
+        <v>77</v>
+      </c>
+      <c r="C10" s="4" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="C11" s="10"/>
+    </row>
+    <row r="12">
+      <c r="C12" s="10"/>
+    </row>
+    <row r="13">
+      <c r="C13" s="10"/>
+    </row>
+    <row r="14">
+      <c r="C14" s="10"/>
+    </row>
+    <row r="15">
+      <c r="C15" s="10"/>
+    </row>
+    <row r="16">
+      <c r="C16" s="10"/>
+    </row>
+    <row r="17">
+      <c r="C17" s="10"/>
+    </row>
+    <row r="18">
+      <c r="C18" s="10"/>
+    </row>
+    <row r="19">
+      <c r="C19" s="10"/>
+    </row>
+    <row r="20">
+      <c r="C20" s="10"/>
+    </row>
+    <row r="21">
+      <c r="C21" s="10"/>
+    </row>
+    <row r="22">
+      <c r="C22" s="10"/>
+    </row>
+    <row r="23">
+      <c r="C23" s="10"/>
+    </row>
+    <row r="24">
+      <c r="C24" s="10"/>
+    </row>
+    <row r="25">
+      <c r="C25" s="10"/>
+    </row>
+    <row r="26">
+      <c r="C26" s="10"/>
+    </row>
+    <row r="27">
+      <c r="C27" s="10"/>
+    </row>
+    <row r="28">
+      <c r="C28" s="10"/>
+    </row>
+    <row r="29">
+      <c r="C29" s="10"/>
+    </row>
+    <row r="30">
+      <c r="C30" s="10"/>
+    </row>
+    <row r="31">
+      <c r="C31" s="10"/>
+    </row>
+    <row r="32">
+      <c r="C32" s="10"/>
+    </row>
+    <row r="33">
+      <c r="C33" s="10"/>
+    </row>
+    <row r="34">
+      <c r="C34" s="10"/>
+    </row>
+    <row r="35">
+      <c r="C35" s="10"/>
+    </row>
+    <row r="36">
+      <c r="C36" s="10"/>
+    </row>
+    <row r="37">
+      <c r="C37" s="10"/>
+    </row>
+    <row r="38">
+      <c r="C38" s="10"/>
+    </row>
+    <row r="39">
+      <c r="C39" s="10"/>
+    </row>
+    <row r="40">
+      <c r="C40" s="10"/>
+    </row>
+    <row r="41">
+      <c r="C41" s="10"/>
+    </row>
+    <row r="42">
+      <c r="C42" s="10"/>
+    </row>
+    <row r="43">
+      <c r="C43" s="10"/>
+    </row>
+    <row r="44">
+      <c r="C44" s="10"/>
+    </row>
+    <row r="45">
+      <c r="C45" s="10"/>
+    </row>
+    <row r="46">
+      <c r="C46" s="10"/>
+    </row>
+    <row r="47">
+      <c r="C47" s="10"/>
+    </row>
+    <row r="48">
+      <c r="C48" s="10"/>
+    </row>
+    <row r="49">
+      <c r="C49" s="10"/>
+    </row>
+    <row r="50">
+      <c r="C50" s="10"/>
+    </row>
+    <row r="51">
+      <c r="C51" s="10"/>
+    </row>
+    <row r="52">
+      <c r="C52" s="10"/>
+    </row>
+    <row r="53">
+      <c r="C53" s="10"/>
+    </row>
+    <row r="54">
+      <c r="C54" s="10"/>
+    </row>
+    <row r="55">
+      <c r="C55" s="10"/>
+    </row>
+    <row r="56">
+      <c r="C56" s="10"/>
+    </row>
+    <row r="57">
+      <c r="C57" s="10"/>
+    </row>
+    <row r="58">
+      <c r="C58" s="10"/>
+    </row>
+    <row r="59">
+      <c r="C59" s="10"/>
+    </row>
+    <row r="60">
+      <c r="C60" s="10"/>
+    </row>
+    <row r="61">
+      <c r="C61" s="10"/>
+    </row>
+    <row r="62">
+      <c r="C62" s="10"/>
+    </row>
+    <row r="63">
+      <c r="C63" s="10"/>
+    </row>
+    <row r="64">
+      <c r="C64" s="10"/>
+    </row>
+    <row r="65">
+      <c r="C65" s="10"/>
+    </row>
+    <row r="66">
+      <c r="C66" s="10"/>
+    </row>
+    <row r="67">
+      <c r="C67" s="10"/>
+    </row>
+    <row r="68">
+      <c r="C68" s="10"/>
+    </row>
+    <row r="69">
+      <c r="C69" s="10"/>
+    </row>
+    <row r="70">
+      <c r="C70" s="10"/>
+    </row>
+    <row r="71">
+      <c r="C71" s="10"/>
+    </row>
+    <row r="72">
+      <c r="C72" s="10"/>
+    </row>
+    <row r="73">
+      <c r="C73" s="10"/>
+    </row>
+    <row r="74">
+      <c r="C74" s="10"/>
+    </row>
+    <row r="75">
+      <c r="C75" s="10"/>
+    </row>
+    <row r="76">
+      <c r="C76" s="10"/>
+    </row>
+    <row r="77">
+      <c r="C77" s="10"/>
+    </row>
+    <row r="78">
+      <c r="C78" s="10"/>
+    </row>
+    <row r="79">
+      <c r="C79" s="10"/>
+    </row>
+    <row r="80">
+      <c r="C80" s="10"/>
+    </row>
+    <row r="81">
+      <c r="C81" s="10"/>
+    </row>
+    <row r="82">
+      <c r="C82" s="10"/>
+    </row>
+    <row r="83">
+      <c r="C83" s="10"/>
+    </row>
+    <row r="84">
+      <c r="C84" s="10"/>
+    </row>
+    <row r="85">
+      <c r="C85" s="10"/>
+    </row>
+    <row r="86">
+      <c r="C86" s="10"/>
+    </row>
+    <row r="87">
+      <c r="C87" s="10"/>
+    </row>
+    <row r="88">
+      <c r="C88" s="10"/>
+    </row>
+    <row r="89">
+      <c r="C89" s="10"/>
+    </row>
+    <row r="90">
+      <c r="C90" s="10"/>
+    </row>
+    <row r="91">
+      <c r="C91" s="10"/>
+    </row>
+    <row r="92">
+      <c r="C92" s="10"/>
+    </row>
+    <row r="93">
+      <c r="C93" s="10"/>
+    </row>
+    <row r="94">
+      <c r="C94" s="10"/>
+    </row>
+    <row r="95">
+      <c r="C95" s="10"/>
+    </row>
+    <row r="96">
+      <c r="C96" s="10"/>
+    </row>
+    <row r="97">
+      <c r="C97" s="10"/>
+    </row>
+    <row r="98">
+      <c r="C98" s="10"/>
+    </row>
+    <row r="99">
+      <c r="C99" s="10"/>
+    </row>
+    <row r="100">
+      <c r="C100" s="10"/>
+    </row>
+    <row r="101">
+      <c r="C101" s="10"/>
+    </row>
+    <row r="102">
+      <c r="C102" s="10"/>
+    </row>
+    <row r="103">
+      <c r="C103" s="10"/>
+    </row>
+    <row r="104">
+      <c r="C104" s="10"/>
+    </row>
+    <row r="105">
+      <c r="C105" s="10"/>
+    </row>
+    <row r="106">
+      <c r="C106" s="10"/>
+    </row>
+    <row r="107">
+      <c r="C107" s="10"/>
+    </row>
+    <row r="108">
+      <c r="C108" s="10"/>
+    </row>
+    <row r="109">
+      <c r="C109" s="10"/>
+    </row>
+    <row r="110">
+      <c r="C110" s="10"/>
+    </row>
+    <row r="111">
+      <c r="C111" s="10"/>
+    </row>
+    <row r="112">
+      <c r="C112" s="10"/>
+    </row>
+    <row r="113">
+      <c r="C113" s="10"/>
+    </row>
+    <row r="114">
+      <c r="C114" s="10"/>
+    </row>
+    <row r="115">
+      <c r="C115" s="10"/>
+    </row>
+    <row r="116">
+      <c r="C116" s="10"/>
+    </row>
+    <row r="117">
+      <c r="C117" s="10"/>
+    </row>
+    <row r="118">
+      <c r="C118" s="10"/>
+    </row>
+    <row r="119">
+      <c r="C119" s="10"/>
+    </row>
+    <row r="120">
+      <c r="C120" s="10"/>
+    </row>
+    <row r="121">
+      <c r="C121" s="10"/>
+    </row>
+    <row r="122">
+      <c r="C122" s="10"/>
+    </row>
+    <row r="123">
+      <c r="C123" s="10"/>
+    </row>
+    <row r="124">
+      <c r="C124" s="10"/>
+    </row>
+    <row r="125">
+      <c r="C125" s="10"/>
+    </row>
+    <row r="126">
+      <c r="C126" s="10"/>
+    </row>
+    <row r="127">
+      <c r="C127" s="10"/>
+    </row>
+    <row r="128">
+      <c r="C128" s="10"/>
+    </row>
+    <row r="129">
+      <c r="C129" s="10"/>
+    </row>
+    <row r="130">
+      <c r="C130" s="10"/>
+    </row>
+    <row r="131">
+      <c r="C131" s="10"/>
+    </row>
+    <row r="132">
+      <c r="C132" s="10"/>
+    </row>
+    <row r="133">
+      <c r="C133" s="10"/>
+    </row>
+    <row r="134">
+      <c r="C134" s="10"/>
+    </row>
+    <row r="135">
+      <c r="C135" s="10"/>
+    </row>
+    <row r="136">
+      <c r="C136" s="10"/>
+    </row>
+    <row r="137">
+      <c r="C137" s="10"/>
+    </row>
+    <row r="138">
+      <c r="C138" s="10"/>
+    </row>
+    <row r="139">
+      <c r="C139" s="10"/>
+    </row>
+    <row r="140">
+      <c r="C140" s="10"/>
+    </row>
+    <row r="141">
+      <c r="C141" s="10"/>
+    </row>
+    <row r="142">
+      <c r="C142" s="10"/>
+    </row>
+    <row r="143">
+      <c r="C143" s="10"/>
+    </row>
+    <row r="144">
+      <c r="C144" s="10"/>
+    </row>
+    <row r="145">
+      <c r="C145" s="10"/>
+    </row>
+    <row r="146">
+      <c r="C146" s="10"/>
+    </row>
+    <row r="147">
+      <c r="C147" s="10"/>
+    </row>
+    <row r="148">
+      <c r="C148" s="10"/>
+    </row>
+    <row r="149">
+      <c r="C149" s="10"/>
+    </row>
+    <row r="150">
+      <c r="C150" s="10"/>
+    </row>
+    <row r="151">
+      <c r="C151" s="10"/>
+    </row>
+    <row r="152">
+      <c r="C152" s="10"/>
+    </row>
+    <row r="153">
+      <c r="C153" s="10"/>
+    </row>
+    <row r="154">
+      <c r="C154" s="10"/>
+    </row>
+    <row r="155">
+      <c r="C155" s="10"/>
+    </row>
+    <row r="156">
+      <c r="C156" s="10"/>
+    </row>
+    <row r="157">
+      <c r="C157" s="10"/>
+    </row>
+    <row r="158">
+      <c r="C158" s="10"/>
+    </row>
+    <row r="159">
+      <c r="C159" s="10"/>
+    </row>
+    <row r="160">
+      <c r="C160" s="10"/>
+    </row>
+    <row r="161">
+      <c r="C161" s="10"/>
+    </row>
+    <row r="162">
+      <c r="C162" s="10"/>
+    </row>
+    <row r="163">
+      <c r="C163" s="10"/>
+    </row>
+    <row r="164">
+      <c r="C164" s="10"/>
+    </row>
+    <row r="165">
+      <c r="C165" s="10"/>
+    </row>
+    <row r="166">
+      <c r="C166" s="10"/>
+    </row>
+    <row r="167">
+      <c r="C167" s="10"/>
+    </row>
+    <row r="168">
+      <c r="C168" s="10"/>
+    </row>
+    <row r="169">
+      <c r="C169" s="10"/>
+    </row>
+    <row r="170">
+      <c r="C170" s="10"/>
+    </row>
+    <row r="171">
+      <c r="C171" s="10"/>
+    </row>
+    <row r="172">
+      <c r="C172" s="10"/>
+    </row>
+    <row r="173">
+      <c r="C173" s="10"/>
+    </row>
+    <row r="174">
+      <c r="C174" s="10"/>
+    </row>
+    <row r="175">
+      <c r="C175" s="10"/>
+    </row>
+    <row r="176">
+      <c r="C176" s="10"/>
+    </row>
+    <row r="177">
+      <c r="C177" s="10"/>
+    </row>
+    <row r="178">
+      <c r="C178" s="10"/>
+    </row>
+    <row r="179">
+      <c r="C179" s="10"/>
+    </row>
+    <row r="180">
+      <c r="C180" s="10"/>
+    </row>
+    <row r="181">
+      <c r="C181" s="10"/>
+    </row>
+    <row r="182">
+      <c r="C182" s="10"/>
+    </row>
+    <row r="183">
+      <c r="C183" s="10"/>
+    </row>
+    <row r="184">
+      <c r="C184" s="10"/>
+    </row>
+    <row r="185">
+      <c r="C185" s="10"/>
+    </row>
+    <row r="186">
+      <c r="C186" s="10"/>
+    </row>
+    <row r="187">
+      <c r="C187" s="10"/>
+    </row>
+    <row r="188">
+      <c r="C188" s="10"/>
+    </row>
+    <row r="189">
+      <c r="C189" s="10"/>
+    </row>
+    <row r="190">
+      <c r="C190" s="10"/>
+    </row>
+    <row r="191">
+      <c r="C191" s="10"/>
+    </row>
+    <row r="192">
+      <c r="C192" s="10"/>
+    </row>
+    <row r="193">
+      <c r="C193" s="10"/>
+    </row>
+    <row r="194">
+      <c r="C194" s="10"/>
+    </row>
+    <row r="195">
+      <c r="C195" s="10"/>
+    </row>
+    <row r="196">
+      <c r="C196" s="10"/>
+    </row>
+    <row r="197">
+      <c r="C197" s="10"/>
+    </row>
+    <row r="198">
+      <c r="C198" s="10"/>
+    </row>
+    <row r="199">
+      <c r="C199" s="10"/>
+    </row>
+    <row r="200">
+      <c r="C200" s="10"/>
+    </row>
+    <row r="201">
+      <c r="C201" s="10"/>
+    </row>
+    <row r="202">
+      <c r="C202" s="10"/>
+    </row>
+    <row r="203">
+      <c r="C203" s="10"/>
+    </row>
+    <row r="204">
+      <c r="C204" s="10"/>
+    </row>
+    <row r="205">
+      <c r="C205" s="10"/>
+    </row>
+    <row r="206">
+      <c r="C206" s="10"/>
+    </row>
+    <row r="207">
+      <c r="C207" s="10"/>
+    </row>
+    <row r="208">
+      <c r="C208" s="10"/>
+    </row>
+    <row r="209">
+      <c r="C209" s="10"/>
+    </row>
+    <row r="210">
+      <c r="C210" s="10"/>
+    </row>
+    <row r="211">
+      <c r="C211" s="10"/>
+    </row>
+    <row r="212">
+      <c r="C212" s="10"/>
+    </row>
+    <row r="213">
+      <c r="C213" s="10"/>
+    </row>
+    <row r="214">
+      <c r="C214" s="10"/>
+    </row>
+    <row r="215">
+      <c r="C215" s="10"/>
+    </row>
+    <row r="216">
+      <c r="C216" s="10"/>
+    </row>
+    <row r="217">
+      <c r="C217" s="10"/>
+    </row>
+    <row r="218">
+      <c r="C218" s="10"/>
+    </row>
+    <row r="219">
+      <c r="C219" s="10"/>
+    </row>
+    <row r="220">
+      <c r="C220" s="10"/>
+    </row>
+    <row r="221">
+      <c r="C221" s="10"/>
+    </row>
+    <row r="222">
+      <c r="C222" s="10"/>
+    </row>
+    <row r="223">
+      <c r="C223" s="10"/>
+    </row>
+    <row r="224">
+      <c r="C224" s="10"/>
+    </row>
+    <row r="225">
+      <c r="C225" s="10"/>
+    </row>
+    <row r="226">
+      <c r="C226" s="10"/>
+    </row>
+    <row r="227">
+      <c r="C227" s="10"/>
+    </row>
+    <row r="228">
+      <c r="C228" s="10"/>
+    </row>
+    <row r="229">
+      <c r="C229" s="10"/>
+    </row>
+    <row r="230">
+      <c r="C230" s="10"/>
+    </row>
+    <row r="231">
+      <c r="C231" s="10"/>
+    </row>
+    <row r="232">
+      <c r="C232" s="10"/>
+    </row>
+    <row r="233">
+      <c r="C233" s="10"/>
+    </row>
+    <row r="234">
+      <c r="C234" s="10"/>
+    </row>
+    <row r="235">
+      <c r="C235" s="10"/>
+    </row>
+    <row r="236">
+      <c r="C236" s="10"/>
+    </row>
+    <row r="237">
+      <c r="C237" s="10"/>
+    </row>
+    <row r="238">
+      <c r="C238" s="10"/>
+    </row>
+    <row r="239">
+      <c r="C239" s="10"/>
+    </row>
+    <row r="240">
+      <c r="C240" s="10"/>
+    </row>
+    <row r="241">
+      <c r="C241" s="10"/>
+    </row>
+    <row r="242">
+      <c r="C242" s="10"/>
+    </row>
+    <row r="243">
+      <c r="C243" s="10"/>
+    </row>
+    <row r="244">
+      <c r="C244" s="10"/>
+    </row>
+    <row r="245">
+      <c r="C245" s="10"/>
+    </row>
+    <row r="246">
+      <c r="C246" s="10"/>
+    </row>
+    <row r="247">
+      <c r="C247" s="10"/>
+    </row>
+    <row r="248">
+      <c r="C248" s="10"/>
+    </row>
+    <row r="249">
+      <c r="C249" s="10"/>
+    </row>
+    <row r="250">
+      <c r="C250" s="10"/>
+    </row>
+    <row r="251">
+      <c r="C251" s="10"/>
+    </row>
+    <row r="252">
+      <c r="C252" s="10"/>
+    </row>
+    <row r="253">
+      <c r="C253" s="10"/>
+    </row>
+    <row r="254">
+      <c r="C254" s="10"/>
+    </row>
+    <row r="255">
+      <c r="C255" s="10"/>
+    </row>
+    <row r="256">
+      <c r="C256" s="10"/>
+    </row>
+    <row r="257">
+      <c r="C257" s="10"/>
+    </row>
+    <row r="258">
+      <c r="C258" s="10"/>
+    </row>
+    <row r="259">
+      <c r="C259" s="10"/>
+    </row>
+    <row r="260">
+      <c r="C260" s="10"/>
+    </row>
+    <row r="261">
+      <c r="C261" s="10"/>
+    </row>
+    <row r="262">
+      <c r="C262" s="10"/>
+    </row>
+    <row r="263">
+      <c r="C263" s="10"/>
+    </row>
+    <row r="264">
+      <c r="C264" s="10"/>
+    </row>
+    <row r="265">
+      <c r="C265" s="10"/>
+    </row>
+    <row r="266">
+      <c r="C266" s="10"/>
+    </row>
+    <row r="267">
+      <c r="C267" s="10"/>
+    </row>
+    <row r="268">
+      <c r="C268" s="10"/>
+    </row>
+    <row r="269">
+      <c r="C269" s="10"/>
+    </row>
+    <row r="270">
+      <c r="C270" s="10"/>
+    </row>
+    <row r="271">
+      <c r="C271" s="10"/>
+    </row>
+    <row r="272">
+      <c r="C272" s="10"/>
+    </row>
+    <row r="273">
+      <c r="C273" s="10"/>
+    </row>
+    <row r="274">
+      <c r="C274" s="10"/>
+    </row>
+    <row r="275">
+      <c r="C275" s="10"/>
+    </row>
+    <row r="276">
+      <c r="C276" s="10"/>
+    </row>
+    <row r="277">
+      <c r="C277" s="10"/>
+    </row>
+    <row r="278">
+      <c r="C278" s="10"/>
+    </row>
+    <row r="279">
+      <c r="C279" s="10"/>
+    </row>
+    <row r="280">
+      <c r="C280" s="10"/>
+    </row>
+    <row r="281">
+      <c r="C281" s="10"/>
+    </row>
+    <row r="282">
+      <c r="C282" s="10"/>
+    </row>
+    <row r="283">
+      <c r="C283" s="10"/>
+    </row>
+    <row r="284">
+      <c r="C284" s="10"/>
+    </row>
+    <row r="285">
+      <c r="C285" s="10"/>
+    </row>
+    <row r="286">
+      <c r="C286" s="10"/>
+    </row>
+    <row r="287">
+      <c r="C287" s="10"/>
+    </row>
+    <row r="288">
+      <c r="C288" s="10"/>
+    </row>
+    <row r="289">
+      <c r="C289" s="10"/>
+    </row>
+    <row r="290">
+      <c r="C290" s="10"/>
+    </row>
+    <row r="291">
+      <c r="C291" s="10"/>
+    </row>
+    <row r="292">
+      <c r="C292" s="10"/>
+    </row>
+    <row r="293">
+      <c r="C293" s="10"/>
+    </row>
+    <row r="294">
+      <c r="C294" s="10"/>
+    </row>
+    <row r="295">
+      <c r="C295" s="10"/>
+    </row>
+    <row r="296">
+      <c r="C296" s="10"/>
+    </row>
+    <row r="297">
+      <c r="C297" s="10"/>
+    </row>
+    <row r="298">
+      <c r="C298" s="10"/>
+    </row>
+    <row r="299">
+      <c r="C299" s="10"/>
+    </row>
+    <row r="300">
+      <c r="C300" s="10"/>
+    </row>
+    <row r="301">
+      <c r="C301" s="10"/>
+    </row>
+    <row r="302">
+      <c r="C302" s="10"/>
+    </row>
+    <row r="303">
+      <c r="C303" s="10"/>
+    </row>
+    <row r="304">
+      <c r="C304" s="10"/>
+    </row>
+    <row r="305">
+      <c r="C305" s="10"/>
+    </row>
+    <row r="306">
+      <c r="C306" s="10"/>
+    </row>
+    <row r="307">
+      <c r="C307" s="10"/>
+    </row>
+    <row r="308">
+      <c r="C308" s="10"/>
+    </row>
+    <row r="309">
+      <c r="C309" s="10"/>
+    </row>
+    <row r="310">
+      <c r="C310" s="10"/>
+    </row>
+    <row r="311">
+      <c r="C311" s="10"/>
+    </row>
+    <row r="312">
+      <c r="C312" s="10"/>
+    </row>
+    <row r="313">
+      <c r="C313" s="10"/>
+    </row>
+    <row r="314">
+      <c r="C314" s="10"/>
+    </row>
+    <row r="315">
+      <c r="C315" s="10"/>
+    </row>
+    <row r="316">
+      <c r="C316" s="10"/>
+    </row>
+    <row r="317">
+      <c r="C317" s="10"/>
+    </row>
+    <row r="318">
+      <c r="C318" s="10"/>
+    </row>
+    <row r="319">
+      <c r="C319" s="10"/>
+    </row>
+    <row r="320">
+      <c r="C320" s="10"/>
+    </row>
+    <row r="321">
+      <c r="C321" s="10"/>
+    </row>
+    <row r="322">
+      <c r="C322" s="10"/>
+    </row>
+    <row r="323">
+      <c r="C323" s="10"/>
+    </row>
+    <row r="324">
+      <c r="C324" s="10"/>
+    </row>
+    <row r="325">
+      <c r="C325" s="10"/>
+    </row>
+    <row r="326">
+      <c r="C326" s="10"/>
+    </row>
+    <row r="327">
+      <c r="C327" s="10"/>
+    </row>
+    <row r="328">
+      <c r="C328" s="10"/>
+    </row>
+    <row r="329">
+      <c r="C329" s="10"/>
+    </row>
+    <row r="330">
+      <c r="C330" s="10"/>
+    </row>
+    <row r="331">
+      <c r="C331" s="10"/>
+    </row>
+    <row r="332">
+      <c r="C332" s="10"/>
+    </row>
+    <row r="333">
+      <c r="C333" s="10"/>
+    </row>
+    <row r="334">
+      <c r="C334" s="10"/>
+    </row>
+    <row r="335">
+      <c r="C335" s="10"/>
+    </row>
+    <row r="336">
+      <c r="C336" s="10"/>
+    </row>
+    <row r="337">
+      <c r="C337" s="10"/>
+    </row>
+    <row r="338">
+      <c r="C338" s="10"/>
+    </row>
+    <row r="339">
+      <c r="C339" s="10"/>
+    </row>
+    <row r="340">
+      <c r="C340" s="10"/>
+    </row>
+    <row r="341">
+      <c r="C341" s="10"/>
+    </row>
+    <row r="342">
+      <c r="C342" s="10"/>
+    </row>
+    <row r="343">
+      <c r="C343" s="10"/>
+    </row>
+    <row r="344">
+      <c r="C344" s="10"/>
+    </row>
+    <row r="345">
+      <c r="C345" s="10"/>
+    </row>
+    <row r="346">
+      <c r="C346" s="10"/>
+    </row>
+    <row r="347">
+      <c r="C347" s="10"/>
+    </row>
+    <row r="348">
+      <c r="C348" s="10"/>
+    </row>
+    <row r="349">
+      <c r="C349" s="10"/>
+    </row>
+    <row r="350">
+      <c r="C350" s="10"/>
+    </row>
+    <row r="351">
+      <c r="C351" s="10"/>
+    </row>
+    <row r="352">
+      <c r="C352" s="10"/>
+    </row>
+    <row r="353">
+      <c r="C353" s="10"/>
+    </row>
+    <row r="354">
+      <c r="C354" s="10"/>
+    </row>
+    <row r="355">
+      <c r="C355" s="10"/>
+    </row>
+    <row r="356">
+      <c r="C356" s="10"/>
+    </row>
+    <row r="357">
+      <c r="C357" s="10"/>
+    </row>
+    <row r="358">
+      <c r="C358" s="10"/>
+    </row>
+    <row r="359">
+      <c r="C359" s="10"/>
+    </row>
+    <row r="360">
+      <c r="C360" s="10"/>
+    </row>
+    <row r="361">
+      <c r="C361" s="10"/>
+    </row>
+    <row r="362">
+      <c r="C362" s="10"/>
+    </row>
+    <row r="363">
+      <c r="C363" s="10"/>
+    </row>
+    <row r="364">
+      <c r="C364" s="10"/>
+    </row>
+    <row r="365">
+      <c r="C365" s="10"/>
+    </row>
+    <row r="366">
+      <c r="C366" s="10"/>
+    </row>
+    <row r="367">
+      <c r="C367" s="10"/>
+    </row>
+    <row r="368">
+      <c r="C368" s="10"/>
+    </row>
+    <row r="369">
+      <c r="C369" s="10"/>
+    </row>
+    <row r="370">
+      <c r="C370" s="10"/>
+    </row>
+    <row r="371">
+      <c r="C371" s="10"/>
+    </row>
+    <row r="372">
+      <c r="C372" s="10"/>
+    </row>
+    <row r="373">
+      <c r="C373" s="10"/>
+    </row>
+    <row r="374">
+      <c r="C374" s="10"/>
+    </row>
+    <row r="375">
+      <c r="C375" s="10"/>
+    </row>
+    <row r="376">
+      <c r="C376" s="10"/>
+    </row>
+    <row r="377">
+      <c r="C377" s="10"/>
+    </row>
+    <row r="378">
+      <c r="C378" s="10"/>
+    </row>
+    <row r="379">
+      <c r="C379" s="10"/>
+    </row>
+    <row r="380">
+      <c r="C380" s="10"/>
+    </row>
+    <row r="381">
+      <c r="C381" s="10"/>
+    </row>
+    <row r="382">
+      <c r="C382" s="10"/>
+    </row>
+    <row r="383">
+      <c r="C383" s="10"/>
+    </row>
+    <row r="384">
+      <c r="C384" s="10"/>
+    </row>
+    <row r="385">
+      <c r="C385" s="10"/>
+    </row>
+    <row r="386">
+      <c r="C386" s="10"/>
+    </row>
+    <row r="387">
+      <c r="C387" s="10"/>
+    </row>
+    <row r="388">
+      <c r="C388" s="10"/>
+    </row>
+    <row r="389">
+      <c r="C389" s="10"/>
+    </row>
+    <row r="390">
+      <c r="C390" s="10"/>
+    </row>
+    <row r="391">
+      <c r="C391" s="10"/>
+    </row>
+    <row r="392">
+      <c r="C392" s="10"/>
+    </row>
+    <row r="393">
+      <c r="C393" s="10"/>
+    </row>
+    <row r="394">
+      <c r="C394" s="10"/>
+    </row>
+    <row r="395">
+      <c r="C395" s="10"/>
+    </row>
+    <row r="396">
+      <c r="C396" s="10"/>
+    </row>
+    <row r="397">
+      <c r="C397" s="10"/>
+    </row>
+    <row r="398">
+      <c r="C398" s="10"/>
+    </row>
+    <row r="399">
+      <c r="C399" s="10"/>
+    </row>
+    <row r="400">
+      <c r="C400" s="10"/>
+    </row>
+    <row r="401">
+      <c r="C401" s="10"/>
+    </row>
+    <row r="402">
+      <c r="C402" s="10"/>
+    </row>
+    <row r="403">
+      <c r="C403" s="10"/>
+    </row>
+    <row r="404">
+      <c r="C404" s="10"/>
+    </row>
+    <row r="405">
+      <c r="C405" s="10"/>
+    </row>
+    <row r="406">
+      <c r="C406" s="10"/>
+    </row>
+    <row r="407">
+      <c r="C407" s="10"/>
+    </row>
+    <row r="408">
+      <c r="C408" s="10"/>
+    </row>
+    <row r="409">
+      <c r="C409" s="10"/>
+    </row>
+    <row r="410">
+      <c r="C410" s="10"/>
+    </row>
+    <row r="411">
+      <c r="C411" s="10"/>
+    </row>
+    <row r="412">
+      <c r="C412" s="10"/>
+    </row>
+    <row r="413">
+      <c r="C413" s="10"/>
+    </row>
+    <row r="414">
+      <c r="C414" s="10"/>
+    </row>
+    <row r="415">
+      <c r="C415" s="10"/>
+    </row>
+    <row r="416">
+      <c r="C416" s="10"/>
+    </row>
+    <row r="417">
+      <c r="C417" s="10"/>
+    </row>
+    <row r="418">
+      <c r="C418" s="10"/>
+    </row>
+    <row r="419">
+      <c r="C419" s="10"/>
+    </row>
+    <row r="420">
+      <c r="C420" s="10"/>
+    </row>
+    <row r="421">
+      <c r="C421" s="10"/>
+    </row>
+    <row r="422">
+      <c r="C422" s="10"/>
+    </row>
+    <row r="423">
+      <c r="C423" s="10"/>
+    </row>
+    <row r="424">
+      <c r="C424" s="10"/>
+    </row>
+    <row r="425">
+      <c r="C425" s="10"/>
+    </row>
+    <row r="426">
+      <c r="C426" s="10"/>
+    </row>
+    <row r="427">
+      <c r="C427" s="10"/>
+    </row>
+    <row r="428">
+      <c r="C428" s="10"/>
+    </row>
+    <row r="429">
+      <c r="C429" s="10"/>
+    </row>
+    <row r="430">
+      <c r="C430" s="10"/>
+    </row>
+    <row r="431">
+      <c r="C431" s="10"/>
+    </row>
+    <row r="432">
+      <c r="C432" s="10"/>
+    </row>
+    <row r="433">
+      <c r="C433" s="10"/>
+    </row>
+    <row r="434">
+      <c r="C434" s="10"/>
+    </row>
+    <row r="435">
+      <c r="C435" s="10"/>
+    </row>
+    <row r="436">
+      <c r="C436" s="10"/>
+    </row>
+    <row r="437">
+      <c r="C437" s="10"/>
+    </row>
+    <row r="438">
+      <c r="C438" s="10"/>
+    </row>
+    <row r="439">
+      <c r="C439" s="10"/>
+    </row>
+    <row r="440">
+      <c r="C440" s="10"/>
+    </row>
+    <row r="441">
+      <c r="C441" s="10"/>
+    </row>
+    <row r="442">
+      <c r="C442" s="10"/>
+    </row>
+    <row r="443">
+      <c r="C443" s="10"/>
+    </row>
+    <row r="444">
+      <c r="C444" s="10"/>
+    </row>
+    <row r="445">
+      <c r="C445" s="10"/>
+    </row>
+    <row r="446">
+      <c r="C446" s="10"/>
+    </row>
+    <row r="447">
+      <c r="C447" s="10"/>
+    </row>
+    <row r="448">
+      <c r="C448" s="10"/>
+    </row>
+    <row r="449">
+      <c r="C449" s="10"/>
+    </row>
+    <row r="450">
+      <c r="C450" s="10"/>
+    </row>
+    <row r="451">
+      <c r="C451" s="10"/>
+    </row>
+    <row r="452">
+      <c r="C452" s="10"/>
+    </row>
+    <row r="453">
+      <c r="C453" s="10"/>
+    </row>
+    <row r="454">
+      <c r="C454" s="10"/>
+    </row>
+    <row r="455">
+      <c r="C455" s="10"/>
+    </row>
+    <row r="456">
+      <c r="C456" s="10"/>
+    </row>
+    <row r="457">
+      <c r="C457" s="10"/>
+    </row>
+    <row r="458">
+      <c r="C458" s="10"/>
+    </row>
+    <row r="459">
+      <c r="C459" s="10"/>
+    </row>
+    <row r="460">
+      <c r="C460" s="10"/>
+    </row>
+    <row r="461">
+      <c r="C461" s="10"/>
+    </row>
+    <row r="462">
+      <c r="C462" s="10"/>
+    </row>
+    <row r="463">
+      <c r="C463" s="10"/>
+    </row>
+    <row r="464">
+      <c r="C464" s="10"/>
+    </row>
+    <row r="465">
+      <c r="C465" s="10"/>
+    </row>
+    <row r="466">
+      <c r="C466" s="10"/>
+    </row>
+    <row r="467">
+      <c r="C467" s="10"/>
+    </row>
+    <row r="468">
+      <c r="C468" s="10"/>
+    </row>
+    <row r="469">
+      <c r="C469" s="10"/>
+    </row>
+    <row r="470">
+      <c r="C470" s="10"/>
+    </row>
+    <row r="471">
+      <c r="C471" s="10"/>
+    </row>
+    <row r="472">
+      <c r="C472" s="10"/>
+    </row>
+    <row r="473">
+      <c r="C473" s="10"/>
+    </row>
+    <row r="474">
+      <c r="C474" s="10"/>
+    </row>
+    <row r="475">
+      <c r="C475" s="10"/>
+    </row>
+    <row r="476">
+      <c r="C476" s="10"/>
+    </row>
+    <row r="477">
+      <c r="C477" s="10"/>
+    </row>
+    <row r="478">
+      <c r="C478" s="10"/>
+    </row>
+    <row r="479">
+      <c r="C479" s="10"/>
+    </row>
+    <row r="480">
+      <c r="C480" s="10"/>
+    </row>
+    <row r="481">
+      <c r="C481" s="10"/>
+    </row>
+    <row r="482">
+      <c r="C482" s="10"/>
+    </row>
+    <row r="483">
+      <c r="C483" s="10"/>
+    </row>
+    <row r="484">
+      <c r="C484" s="10"/>
+    </row>
+    <row r="485">
+      <c r="C485" s="10"/>
+    </row>
+    <row r="486">
+      <c r="C486" s="10"/>
+    </row>
+    <row r="487">
+      <c r="C487" s="10"/>
+    </row>
+    <row r="488">
+      <c r="C488" s="10"/>
+    </row>
+    <row r="489">
+      <c r="C489" s="10"/>
+    </row>
+    <row r="490">
+      <c r="C490" s="10"/>
+    </row>
+    <row r="491">
+      <c r="C491" s="10"/>
+    </row>
+    <row r="492">
+      <c r="C492" s="10"/>
+    </row>
+    <row r="493">
+      <c r="C493" s="10"/>
+    </row>
+    <row r="494">
+      <c r="C494" s="10"/>
+    </row>
+    <row r="495">
+      <c r="C495" s="10"/>
+    </row>
+    <row r="496">
+      <c r="C496" s="10"/>
+    </row>
+    <row r="497">
+      <c r="C497" s="10"/>
+    </row>
+    <row r="498">
+      <c r="C498" s="10"/>
+    </row>
+    <row r="499">
+      <c r="C499" s="10"/>
+    </row>
+    <row r="500">
+      <c r="C500" s="10"/>
+    </row>
+    <row r="501">
+      <c r="C501" s="10"/>
+    </row>
+    <row r="502">
+      <c r="C502" s="10"/>
+    </row>
+    <row r="503">
+      <c r="C503" s="10"/>
+    </row>
+    <row r="504">
+      <c r="C504" s="10"/>
+    </row>
+    <row r="505">
+      <c r="C505" s="10"/>
+    </row>
+    <row r="506">
+      <c r="C506" s="10"/>
+    </row>
+    <row r="507">
+      <c r="C507" s="10"/>
+    </row>
+    <row r="508">
+      <c r="C508" s="10"/>
+    </row>
+    <row r="509">
+      <c r="C509" s="10"/>
+    </row>
+    <row r="510">
+      <c r="C510" s="10"/>
+    </row>
+    <row r="511">
+      <c r="C511" s="10"/>
+    </row>
+    <row r="512">
+      <c r="C512" s="10"/>
+    </row>
+    <row r="513">
+      <c r="C513" s="10"/>
+    </row>
+    <row r="514">
+      <c r="C514" s="10"/>
+    </row>
+    <row r="515">
+      <c r="C515" s="10"/>
+    </row>
+    <row r="516">
+      <c r="C516" s="10"/>
+    </row>
+    <row r="517">
+      <c r="C517" s="10"/>
+    </row>
+    <row r="518">
+      <c r="C518" s="10"/>
+    </row>
+    <row r="519">
+      <c r="C519" s="10"/>
+    </row>
+    <row r="520">
+      <c r="C520" s="10"/>
+    </row>
+    <row r="521">
+      <c r="C521" s="10"/>
+    </row>
+    <row r="522">
+      <c r="C522" s="10"/>
+    </row>
+    <row r="523">
+      <c r="C523" s="10"/>
+    </row>
+    <row r="524">
+      <c r="C524" s="10"/>
+    </row>
+    <row r="525">
+      <c r="C525" s="10"/>
+    </row>
+    <row r="526">
+      <c r="C526" s="10"/>
+    </row>
+    <row r="527">
+      <c r="C527" s="10"/>
+    </row>
+    <row r="528">
+      <c r="C528" s="10"/>
+    </row>
+    <row r="529">
+      <c r="C529" s="10"/>
+    </row>
+    <row r="530">
+      <c r="C530" s="10"/>
+    </row>
+    <row r="531">
+      <c r="C531" s="10"/>
+    </row>
+    <row r="532">
+      <c r="C532" s="10"/>
+    </row>
+    <row r="533">
+      <c r="C533" s="10"/>
+    </row>
+    <row r="534">
+      <c r="C534" s="10"/>
+    </row>
+    <row r="535">
+      <c r="C535" s="10"/>
+    </row>
+    <row r="536">
+      <c r="C536" s="10"/>
+    </row>
+    <row r="537">
+      <c r="C537" s="10"/>
+    </row>
+    <row r="538">
+      <c r="C538" s="10"/>
+    </row>
+    <row r="539">
+      <c r="C539" s="10"/>
+    </row>
+    <row r="540">
+      <c r="C540" s="10"/>
+    </row>
+    <row r="541">
+      <c r="C541" s="10"/>
+    </row>
+    <row r="542">
+      <c r="C542" s="10"/>
+    </row>
+    <row r="543">
+      <c r="C543" s="10"/>
+    </row>
+    <row r="544">
+      <c r="C544" s="10"/>
+    </row>
+    <row r="545">
+      <c r="C545" s="10"/>
+    </row>
+    <row r="546">
+      <c r="C546" s="10"/>
+    </row>
+    <row r="547">
+      <c r="C547" s="10"/>
+    </row>
+    <row r="548">
+      <c r="C548" s="10"/>
+    </row>
+    <row r="549">
+      <c r="C549" s="10"/>
+    </row>
+    <row r="550">
+      <c r="C550" s="10"/>
+    </row>
+    <row r="551">
+      <c r="C551" s="10"/>
+    </row>
+    <row r="552">
+      <c r="C552" s="10"/>
+    </row>
+    <row r="553">
+      <c r="C553" s="10"/>
+    </row>
+    <row r="554">
+      <c r="C554" s="10"/>
+    </row>
+    <row r="555">
+      <c r="C555" s="10"/>
+    </row>
+    <row r="556">
+      <c r="C556" s="10"/>
+    </row>
+    <row r="557">
+      <c r="C557" s="10"/>
+    </row>
+    <row r="558">
+      <c r="C558" s="10"/>
+    </row>
+    <row r="559">
+      <c r="C559" s="10"/>
+    </row>
+    <row r="560">
+      <c r="C560" s="10"/>
+    </row>
+    <row r="561">
+      <c r="C561" s="10"/>
+    </row>
+    <row r="562">
+      <c r="C562" s="10"/>
+    </row>
+    <row r="563">
+      <c r="C563" s="10"/>
+    </row>
+    <row r="564">
+      <c r="C564" s="10"/>
+    </row>
+    <row r="565">
+      <c r="C565" s="10"/>
+    </row>
+    <row r="566">
+      <c r="C566" s="10"/>
+    </row>
+    <row r="567">
+      <c r="C567" s="10"/>
+    </row>
+    <row r="568">
+      <c r="C568" s="10"/>
+    </row>
+    <row r="569">
+      <c r="C569" s="10"/>
+    </row>
+    <row r="570">
+      <c r="C570" s="10"/>
+    </row>
+    <row r="571">
+      <c r="C571" s="10"/>
+    </row>
+    <row r="572">
+      <c r="C572" s="10"/>
+    </row>
+    <row r="573">
+      <c r="C573" s="10"/>
+    </row>
+    <row r="574">
+      <c r="C574" s="10"/>
+    </row>
+    <row r="575">
+      <c r="C575" s="10"/>
+    </row>
+    <row r="576">
+      <c r="C576" s="10"/>
+    </row>
+    <row r="577">
+      <c r="C577" s="10"/>
+    </row>
+    <row r="578">
+      <c r="C578" s="10"/>
+    </row>
+    <row r="579">
+      <c r="C579" s="10"/>
+    </row>
+    <row r="580">
+      <c r="C580" s="10"/>
+    </row>
+    <row r="581">
+      <c r="C581" s="10"/>
+    </row>
+    <row r="582">
+      <c r="C582" s="10"/>
+    </row>
+    <row r="583">
+      <c r="C583" s="10"/>
+    </row>
+    <row r="584">
+      <c r="C584" s="10"/>
+    </row>
+    <row r="585">
+      <c r="C585" s="10"/>
+    </row>
+    <row r="586">
+      <c r="C586" s="10"/>
+    </row>
+    <row r="587">
+      <c r="C587" s="10"/>
+    </row>
+    <row r="588">
+      <c r="C588" s="10"/>
+    </row>
+    <row r="589">
+      <c r="C589" s="10"/>
+    </row>
+    <row r="590">
+      <c r="C590" s="10"/>
+    </row>
+    <row r="591">
+      <c r="C591" s="10"/>
+    </row>
+    <row r="592">
+      <c r="C592" s="10"/>
+    </row>
+    <row r="593">
+      <c r="C593" s="10"/>
+    </row>
+    <row r="594">
+      <c r="C594" s="10"/>
+    </row>
+    <row r="595">
+      <c r="C595" s="10"/>
+    </row>
+    <row r="596">
+      <c r="C596" s="10"/>
+    </row>
+    <row r="597">
+      <c r="C597" s="10"/>
+    </row>
+    <row r="598">
+      <c r="C598" s="10"/>
+    </row>
+    <row r="599">
+      <c r="C599" s="10"/>
+    </row>
+    <row r="600">
+      <c r="C600" s="10"/>
+    </row>
+    <row r="601">
+      <c r="C601" s="10"/>
+    </row>
+    <row r="602">
+      <c r="C602" s="10"/>
+    </row>
+    <row r="603">
+      <c r="C603" s="10"/>
+    </row>
+    <row r="604">
+      <c r="C604" s="10"/>
+    </row>
+    <row r="605">
+      <c r="C605" s="10"/>
+    </row>
+    <row r="606">
+      <c r="C606" s="10"/>
+    </row>
+    <row r="607">
+      <c r="C607" s="10"/>
+    </row>
+    <row r="608">
+      <c r="C608" s="10"/>
+    </row>
+    <row r="609">
+      <c r="C609" s="10"/>
+    </row>
+    <row r="610">
+      <c r="C610" s="10"/>
+    </row>
+    <row r="611">
+      <c r="C611" s="10"/>
+    </row>
+    <row r="612">
+      <c r="C612" s="10"/>
+    </row>
+    <row r="613">
+      <c r="C613" s="10"/>
+    </row>
+    <row r="614">
+      <c r="C614" s="10"/>
+    </row>
+    <row r="615">
+      <c r="C615" s="10"/>
+    </row>
+    <row r="616">
+      <c r="C616" s="10"/>
+    </row>
+    <row r="617">
+      <c r="C617" s="10"/>
+    </row>
+    <row r="618">
+      <c r="C618" s="10"/>
+    </row>
+    <row r="619">
+      <c r="C619" s="10"/>
+    </row>
+    <row r="620">
+      <c r="C620" s="10"/>
+    </row>
+    <row r="621">
+      <c r="C621" s="10"/>
+    </row>
+    <row r="622">
+      <c r="C622" s="10"/>
+    </row>
+    <row r="623">
+      <c r="C623" s="10"/>
+    </row>
+    <row r="624">
+      <c r="C624" s="10"/>
+    </row>
+    <row r="625">
+      <c r="C625" s="10"/>
+    </row>
+    <row r="626">
+      <c r="C626" s="10"/>
+    </row>
+    <row r="627">
+      <c r="C627" s="10"/>
+    </row>
+    <row r="628">
+      <c r="C628" s="10"/>
+    </row>
+    <row r="629">
+      <c r="C629" s="10"/>
+    </row>
+    <row r="630">
+      <c r="C630" s="10"/>
+    </row>
+    <row r="631">
+      <c r="C631" s="10"/>
+    </row>
+    <row r="632">
+      <c r="C632" s="10"/>
+    </row>
+    <row r="633">
+      <c r="C633" s="10"/>
+    </row>
+    <row r="634">
+      <c r="C634" s="10"/>
+    </row>
+    <row r="635">
+      <c r="C635" s="10"/>
+    </row>
+    <row r="636">
+      <c r="C636" s="10"/>
+    </row>
+    <row r="637">
+      <c r="C637" s="10"/>
+    </row>
+    <row r="638">
+      <c r="C638" s="10"/>
+    </row>
+    <row r="639">
+      <c r="C639" s="10"/>
+    </row>
+    <row r="640">
+      <c r="C640" s="10"/>
+    </row>
+    <row r="641">
+      <c r="C641" s="10"/>
+    </row>
+    <row r="642">
+      <c r="C642" s="10"/>
+    </row>
+    <row r="643">
+      <c r="C643" s="10"/>
+    </row>
+    <row r="644">
+      <c r="C644" s="10"/>
+    </row>
+    <row r="645">
+      <c r="C645" s="10"/>
+    </row>
+    <row r="646">
+      <c r="C646" s="10"/>
+    </row>
+    <row r="647">
+      <c r="C647" s="10"/>
+    </row>
+    <row r="648">
+      <c r="C648" s="10"/>
+    </row>
+    <row r="649">
+      <c r="C649" s="10"/>
+    </row>
+    <row r="650">
+      <c r="C650" s="10"/>
+    </row>
+    <row r="651">
+      <c r="C651" s="10"/>
+    </row>
+    <row r="652">
+      <c r="C652" s="10"/>
+    </row>
+    <row r="653">
+      <c r="C653" s="10"/>
+    </row>
+    <row r="654">
+      <c r="C654" s="10"/>
+    </row>
+    <row r="655">
+      <c r="C655" s="10"/>
+    </row>
+    <row r="656">
+      <c r="C656" s="10"/>
+    </row>
+    <row r="657">
+      <c r="C657" s="10"/>
+    </row>
+    <row r="658">
+      <c r="C658" s="10"/>
+    </row>
+    <row r="659">
+      <c r="C659" s="10"/>
+    </row>
+    <row r="660">
+      <c r="C660" s="10"/>
+    </row>
+    <row r="661">
+      <c r="C661" s="10"/>
+    </row>
+    <row r="662">
+      <c r="C662" s="10"/>
+    </row>
+    <row r="663">
+      <c r="C663" s="10"/>
+    </row>
+    <row r="664">
+      <c r="C664" s="10"/>
+    </row>
+    <row r="665">
+      <c r="C665" s="10"/>
+    </row>
+    <row r="666">
+      <c r="C666" s="10"/>
+    </row>
+    <row r="667">
+      <c r="C667" s="10"/>
+    </row>
+    <row r="668">
+      <c r="C668" s="10"/>
+    </row>
+    <row r="669">
+      <c r="C669" s="10"/>
+    </row>
+    <row r="670">
+      <c r="C670" s="10"/>
+    </row>
+    <row r="671">
+      <c r="C671" s="10"/>
+    </row>
+    <row r="672">
+      <c r="C672" s="10"/>
+    </row>
+    <row r="673">
+      <c r="C673" s="10"/>
+    </row>
+    <row r="674">
+      <c r="C674" s="10"/>
+    </row>
+    <row r="675">
+      <c r="C675" s="10"/>
+    </row>
+    <row r="676">
+      <c r="C676" s="10"/>
+    </row>
+    <row r="677">
+      <c r="C677" s="10"/>
+    </row>
+    <row r="678">
+      <c r="C678" s="10"/>
+    </row>
+    <row r="679">
+      <c r="C679" s="10"/>
+    </row>
+    <row r="680">
+      <c r="C680" s="10"/>
+    </row>
+    <row r="681">
+      <c r="C681" s="10"/>
+    </row>
+    <row r="682">
+      <c r="C682" s="10"/>
+    </row>
+    <row r="683">
+      <c r="C683" s="10"/>
+    </row>
+    <row r="684">
+      <c r="C684" s="10"/>
+    </row>
+    <row r="685">
+      <c r="C685" s="10"/>
+    </row>
+    <row r="686">
+      <c r="C686" s="10"/>
+    </row>
+    <row r="687">
+      <c r="C687" s="10"/>
+    </row>
+    <row r="688">
+      <c r="C688" s="10"/>
+    </row>
+    <row r="689">
+      <c r="C689" s="10"/>
+    </row>
+    <row r="690">
+      <c r="C690" s="10"/>
+    </row>
+    <row r="691">
+      <c r="C691" s="10"/>
+    </row>
+    <row r="692">
+      <c r="C692" s="10"/>
+    </row>
+    <row r="693">
+      <c r="C693" s="10"/>
+    </row>
+    <row r="694">
+      <c r="C694" s="10"/>
+    </row>
+    <row r="695">
+      <c r="C695" s="10"/>
+    </row>
+    <row r="696">
+      <c r="C696" s="10"/>
+    </row>
+    <row r="697">
+      <c r="C697" s="10"/>
+    </row>
+    <row r="698">
+      <c r="C698" s="10"/>
+    </row>
+    <row r="699">
+      <c r="C699" s="10"/>
+    </row>
+    <row r="700">
+      <c r="C700" s="10"/>
+    </row>
+    <row r="701">
+      <c r="C701" s="10"/>
+    </row>
+    <row r="702">
+      <c r="C702" s="10"/>
+    </row>
+    <row r="703">
+      <c r="C703" s="10"/>
+    </row>
+    <row r="704">
+      <c r="C704" s="10"/>
+    </row>
+    <row r="705">
+      <c r="C705" s="10"/>
+    </row>
+    <row r="706">
+      <c r="C706" s="10"/>
+    </row>
+    <row r="707">
+      <c r="C707" s="10"/>
+    </row>
+    <row r="708">
+      <c r="C708" s="10"/>
+    </row>
+    <row r="709">
+      <c r="C709" s="10"/>
+    </row>
+    <row r="710">
+      <c r="C710" s="10"/>
+    </row>
+    <row r="711">
+      <c r="C711" s="10"/>
+    </row>
+    <row r="712">
+      <c r="C712" s="10"/>
+    </row>
+    <row r="713">
+      <c r="C713" s="10"/>
+    </row>
+    <row r="714">
+      <c r="C714" s="10"/>
+    </row>
+    <row r="715">
+      <c r="C715" s="10"/>
+    </row>
+    <row r="716">
+      <c r="C716" s="10"/>
+    </row>
+    <row r="717">
+      <c r="C717" s="10"/>
+    </row>
+    <row r="718">
+      <c r="C718" s="10"/>
+    </row>
+    <row r="719">
+      <c r="C719" s="10"/>
+    </row>
+    <row r="720">
+      <c r="C720" s="10"/>
+    </row>
+    <row r="721">
+      <c r="C721" s="10"/>
+    </row>
+    <row r="722">
+      <c r="C722" s="10"/>
+    </row>
+    <row r="723">
+      <c r="C723" s="10"/>
+    </row>
+    <row r="724">
+      <c r="C724" s="10"/>
+    </row>
+    <row r="725">
+      <c r="C725" s="10"/>
+    </row>
+    <row r="726">
+      <c r="C726" s="10"/>
+    </row>
+    <row r="727">
+      <c r="C727" s="10"/>
+    </row>
+    <row r="728">
+      <c r="C728" s="10"/>
+    </row>
+    <row r="729">
+      <c r="C729" s="10"/>
+    </row>
+    <row r="730">
+      <c r="C730" s="10"/>
+    </row>
+    <row r="731">
+      <c r="C731" s="10"/>
+    </row>
+    <row r="732">
+      <c r="C732" s="10"/>
+    </row>
+    <row r="733">
+      <c r="C733" s="10"/>
+    </row>
+    <row r="734">
+      <c r="C734" s="10"/>
+    </row>
+    <row r="735">
+      <c r="C735" s="10"/>
+    </row>
+    <row r="736">
+      <c r="C736" s="10"/>
+    </row>
+    <row r="737">
+      <c r="C737" s="10"/>
+    </row>
+    <row r="738">
+      <c r="C738" s="10"/>
+    </row>
+    <row r="739">
+      <c r="C739" s="10"/>
+    </row>
+    <row r="740">
+      <c r="C740" s="10"/>
+    </row>
+    <row r="741">
+      <c r="C741" s="10"/>
+    </row>
+    <row r="742">
+      <c r="C742" s="10"/>
+    </row>
+    <row r="743">
+      <c r="C743" s="10"/>
+    </row>
+    <row r="744">
+      <c r="C744" s="10"/>
+    </row>
+    <row r="745">
+      <c r="C745" s="10"/>
+    </row>
+    <row r="746">
+      <c r="C746" s="10"/>
+    </row>
+    <row r="747">
+      <c r="C747" s="10"/>
+    </row>
+    <row r="748">
+      <c r="C748" s="10"/>
+    </row>
+    <row r="749">
+      <c r="C749" s="10"/>
+    </row>
+    <row r="750">
+      <c r="C750" s="10"/>
+    </row>
+    <row r="751">
+      <c r="C751" s="10"/>
+    </row>
+    <row r="752">
+      <c r="C752" s="10"/>
+    </row>
+    <row r="753">
+      <c r="C753" s="10"/>
+    </row>
+    <row r="754">
+      <c r="C754" s="10"/>
+    </row>
+    <row r="755">
+      <c r="C755" s="10"/>
+    </row>
+    <row r="756">
+      <c r="C756" s="10"/>
+    </row>
+    <row r="757">
+      <c r="C757" s="10"/>
+    </row>
+    <row r="758">
+      <c r="C758" s="10"/>
+    </row>
+    <row r="759">
+      <c r="C759" s="10"/>
+    </row>
+    <row r="760">
+      <c r="C760" s="10"/>
+    </row>
+    <row r="761">
+      <c r="C761" s="10"/>
+    </row>
+    <row r="762">
+      <c r="C762" s="10"/>
+    </row>
+    <row r="763">
+      <c r="C763" s="10"/>
+    </row>
+    <row r="764">
+      <c r="C764" s="10"/>
+    </row>
+    <row r="765">
+      <c r="C765" s="10"/>
+    </row>
+    <row r="766">
+      <c r="C766" s="10"/>
+    </row>
+    <row r="767">
+      <c r="C767" s="10"/>
+    </row>
+    <row r="768">
+      <c r="C768" s="10"/>
+    </row>
+    <row r="769">
+      <c r="C769" s="10"/>
+    </row>
+    <row r="770">
+      <c r="C770" s="10"/>
+    </row>
+    <row r="771">
+      <c r="C771" s="10"/>
+    </row>
+    <row r="772">
+      <c r="C772" s="10"/>
+    </row>
+    <row r="773">
+      <c r="C773" s="10"/>
+    </row>
+    <row r="774">
+      <c r="C774" s="10"/>
+    </row>
+    <row r="775">
+      <c r="C775" s="10"/>
+    </row>
+    <row r="776">
+      <c r="C776" s="10"/>
+    </row>
+    <row r="777">
+      <c r="C777" s="10"/>
+    </row>
+    <row r="778">
+      <c r="C778" s="10"/>
+    </row>
+    <row r="779">
+      <c r="C779" s="10"/>
+    </row>
+    <row r="780">
+      <c r="C780" s="10"/>
+    </row>
+    <row r="781">
+      <c r="C781" s="10"/>
+    </row>
+    <row r="782">
+      <c r="C782" s="10"/>
+    </row>
+    <row r="783">
+      <c r="C783" s="10"/>
+    </row>
+    <row r="784">
+      <c r="C784" s="10"/>
+    </row>
+    <row r="785">
+      <c r="C785" s="10"/>
+    </row>
+    <row r="786">
+      <c r="C786" s="10"/>
+    </row>
+    <row r="787">
+      <c r="C787" s="10"/>
+    </row>
+    <row r="788">
+      <c r="C788" s="10"/>
+    </row>
+    <row r="789">
+      <c r="C789" s="10"/>
+    </row>
+    <row r="790">
+      <c r="C790" s="10"/>
+    </row>
+    <row r="791">
+      <c r="C791" s="10"/>
+    </row>
+    <row r="792">
+      <c r="C792" s="10"/>
+    </row>
+    <row r="793">
+      <c r="C793" s="10"/>
+    </row>
+    <row r="794">
+      <c r="C794" s="10"/>
+    </row>
+    <row r="795">
+      <c r="C795" s="10"/>
+    </row>
+    <row r="796">
+      <c r="C796" s="10"/>
+    </row>
+    <row r="797">
+      <c r="C797" s="10"/>
+    </row>
+    <row r="798">
+      <c r="C798" s="10"/>
+    </row>
+    <row r="799">
+      <c r="C799" s="10"/>
+    </row>
+    <row r="800">
+      <c r="C800" s="10"/>
+    </row>
+    <row r="801">
+      <c r="C801" s="10"/>
+    </row>
+    <row r="802">
+      <c r="C802" s="10"/>
+    </row>
+    <row r="803">
+      <c r="C803" s="10"/>
+    </row>
+    <row r="804">
+      <c r="C804" s="10"/>
+    </row>
+    <row r="805">
+      <c r="C805" s="10"/>
+    </row>
+    <row r="806">
+      <c r="C806" s="10"/>
+    </row>
+    <row r="807">
+      <c r="C807" s="10"/>
+    </row>
+    <row r="808">
+      <c r="C808" s="10"/>
+    </row>
+    <row r="809">
+      <c r="C809" s="10"/>
+    </row>
+    <row r="810">
+      <c r="C810" s="10"/>
+    </row>
+    <row r="811">
+      <c r="C811" s="10"/>
+    </row>
+    <row r="812">
+      <c r="C812" s="10"/>
+    </row>
+    <row r="813">
+      <c r="C813" s="10"/>
+    </row>
+    <row r="814">
+      <c r="C814" s="10"/>
+    </row>
+    <row r="815">
+      <c r="C815" s="10"/>
+    </row>
+    <row r="816">
+      <c r="C816" s="10"/>
+    </row>
+    <row r="817">
+      <c r="C817" s="10"/>
+    </row>
+    <row r="818">
+      <c r="C818" s="10"/>
+    </row>
+    <row r="819">
+      <c r="C819" s="10"/>
+    </row>
+    <row r="820">
+      <c r="C820" s="10"/>
+    </row>
+    <row r="821">
+      <c r="C821" s="10"/>
+    </row>
+    <row r="822">
+      <c r="C822" s="10"/>
+    </row>
+    <row r="823">
+      <c r="C823" s="10"/>
+    </row>
+    <row r="824">
+      <c r="C824" s="10"/>
+    </row>
+    <row r="825">
+      <c r="C825" s="10"/>
+    </row>
+    <row r="826">
+      <c r="C826" s="10"/>
+    </row>
+    <row r="827">
+      <c r="C827" s="10"/>
+    </row>
+    <row r="828">
+      <c r="C828" s="10"/>
+    </row>
+    <row r="829">
+      <c r="C829" s="10"/>
+    </row>
+    <row r="830">
+      <c r="C830" s="10"/>
+    </row>
+    <row r="831">
+      <c r="C831" s="10"/>
+    </row>
+    <row r="832">
+      <c r="C832" s="10"/>
+    </row>
+    <row r="833">
+      <c r="C833" s="10"/>
+    </row>
+    <row r="834">
+      <c r="C834" s="10"/>
+    </row>
+    <row r="835">
+      <c r="C835" s="10"/>
+    </row>
+    <row r="836">
+      <c r="C836" s="10"/>
+    </row>
+    <row r="837">
+      <c r="C837" s="10"/>
+    </row>
+    <row r="838">
+      <c r="C838" s="10"/>
+    </row>
+    <row r="839">
+      <c r="C839" s="10"/>
+    </row>
+    <row r="840">
+      <c r="C840" s="10"/>
+    </row>
+    <row r="841">
+      <c r="C841" s="10"/>
+    </row>
+    <row r="842">
+      <c r="C842" s="10"/>
+    </row>
+    <row r="843">
+      <c r="C843" s="10"/>
+    </row>
+    <row r="844">
+      <c r="C844" s="10"/>
+    </row>
+    <row r="845">
+      <c r="C845" s="10"/>
+    </row>
+    <row r="846">
+      <c r="C846" s="10"/>
+    </row>
+    <row r="847">
+      <c r="C847" s="10"/>
+    </row>
+    <row r="848">
+      <c r="C848" s="10"/>
+    </row>
+    <row r="849">
+      <c r="C849" s="10"/>
+    </row>
+    <row r="850">
+      <c r="C850" s="10"/>
+    </row>
+    <row r="851">
+      <c r="C851" s="10"/>
+    </row>
+    <row r="852">
+      <c r="C852" s="10"/>
+    </row>
+    <row r="853">
+      <c r="C853" s="10"/>
+    </row>
+    <row r="854">
+      <c r="C854" s="10"/>
+    </row>
+    <row r="855">
+      <c r="C855" s="10"/>
+    </row>
+    <row r="856">
+      <c r="C856" s="10"/>
+    </row>
+    <row r="857">
+      <c r="C857" s="10"/>
+    </row>
+    <row r="858">
+      <c r="C858" s="10"/>
+    </row>
+    <row r="859">
+      <c r="C859" s="10"/>
+    </row>
+    <row r="860">
+      <c r="C860" s="10"/>
+    </row>
+    <row r="861">
+      <c r="C861" s="10"/>
+    </row>
+    <row r="862">
+      <c r="C862" s="10"/>
+    </row>
+    <row r="863">
+      <c r="C863" s="10"/>
+    </row>
+    <row r="864">
+      <c r="C864" s="10"/>
+    </row>
+    <row r="865">
+      <c r="C865" s="10"/>
+    </row>
+    <row r="866">
+      <c r="C866" s="10"/>
+    </row>
+    <row r="867">
+      <c r="C867" s="10"/>
+    </row>
+    <row r="868">
+      <c r="C868" s="10"/>
+    </row>
+    <row r="869">
+      <c r="C869" s="10"/>
+    </row>
+    <row r="870">
+      <c r="C870" s="10"/>
+    </row>
+    <row r="871">
+      <c r="C871" s="10"/>
+    </row>
+    <row r="872">
+      <c r="C872" s="10"/>
+    </row>
+    <row r="873">
+      <c r="C873" s="10"/>
+    </row>
+    <row r="874">
+      <c r="C874" s="10"/>
+    </row>
+    <row r="875">
+      <c r="C875" s="10"/>
+    </row>
+    <row r="876">
+      <c r="C876" s="10"/>
+    </row>
+    <row r="877">
+      <c r="C877" s="10"/>
+    </row>
+    <row r="878">
+      <c r="C878" s="10"/>
+    </row>
+    <row r="879">
+      <c r="C879" s="10"/>
+    </row>
+    <row r="880">
+      <c r="C880" s="10"/>
+    </row>
+    <row r="881">
+      <c r="C881" s="10"/>
+    </row>
+    <row r="882">
+      <c r="C882" s="10"/>
+    </row>
+    <row r="883">
+      <c r="C883" s="10"/>
+    </row>
+    <row r="884">
+      <c r="C884" s="10"/>
+    </row>
+    <row r="885">
+      <c r="C885" s="10"/>
+    </row>
+    <row r="886">
+      <c r="C886" s="10"/>
+    </row>
+    <row r="887">
+      <c r="C887" s="10"/>
+    </row>
+    <row r="888">
+      <c r="C888" s="10"/>
+    </row>
+    <row r="889">
+      <c r="C889" s="10"/>
+    </row>
+    <row r="890">
+      <c r="C890" s="10"/>
+    </row>
+    <row r="891">
+      <c r="C891" s="10"/>
+    </row>
+    <row r="892">
+      <c r="C892" s="10"/>
+    </row>
+    <row r="893">
+      <c r="C893" s="10"/>
+    </row>
+    <row r="894">
+      <c r="C894" s="10"/>
+    </row>
+    <row r="895">
+      <c r="C895" s="10"/>
+    </row>
+    <row r="896">
+      <c r="C896" s="10"/>
+    </row>
+    <row r="897">
+      <c r="C897" s="10"/>
+    </row>
+    <row r="898">
+      <c r="C898" s="10"/>
+    </row>
+    <row r="899">
+      <c r="C899" s="10"/>
+    </row>
+    <row r="900">
+      <c r="C900" s="10"/>
+    </row>
+    <row r="901">
+      <c r="C901" s="10"/>
+    </row>
+    <row r="902">
+      <c r="C902" s="10"/>
+    </row>
+    <row r="903">
+      <c r="C903" s="10"/>
+    </row>
+    <row r="904">
+      <c r="C904" s="10"/>
+    </row>
+    <row r="905">
+      <c r="C905" s="10"/>
+    </row>
+    <row r="906">
+      <c r="C906" s="10"/>
+    </row>
+    <row r="907">
+      <c r="C907" s="10"/>
+    </row>
+    <row r="908">
+      <c r="C908" s="10"/>
+    </row>
+    <row r="909">
+      <c r="C909" s="10"/>
+    </row>
+    <row r="910">
+      <c r="C910" s="10"/>
+    </row>
+    <row r="911">
+      <c r="C911" s="10"/>
+    </row>
+    <row r="912">
+      <c r="C912" s="10"/>
+    </row>
+    <row r="913">
+      <c r="C913" s="10"/>
+    </row>
+    <row r="914">
+      <c r="C914" s="10"/>
+    </row>
+    <row r="915">
+      <c r="C915" s="10"/>
+    </row>
+    <row r="916">
+      <c r="C916" s="10"/>
+    </row>
+    <row r="917">
+      <c r="C917" s="10"/>
+    </row>
+    <row r="918">
+      <c r="C918" s="10"/>
+    </row>
+    <row r="919">
+      <c r="C919" s="10"/>
+    </row>
+    <row r="920">
+      <c r="C920" s="10"/>
+    </row>
+    <row r="921">
+      <c r="C921" s="10"/>
+    </row>
+    <row r="922">
+      <c r="C922" s="10"/>
+    </row>
+    <row r="923">
+      <c r="C923" s="10"/>
+    </row>
+    <row r="924">
+      <c r="C924" s="10"/>
+    </row>
+    <row r="925">
+      <c r="C925" s="10"/>
+    </row>
+    <row r="926">
+      <c r="C926" s="10"/>
+    </row>
+    <row r="927">
+      <c r="C927" s="10"/>
+    </row>
+    <row r="928">
+      <c r="C928" s="10"/>
+    </row>
+    <row r="929">
+      <c r="C929" s="10"/>
+    </row>
+    <row r="930">
+      <c r="C930" s="10"/>
+    </row>
+    <row r="931">
+      <c r="C931" s="10"/>
+    </row>
+    <row r="932">
+      <c r="C932" s="10"/>
+    </row>
+    <row r="933">
+      <c r="C933" s="10"/>
+    </row>
+    <row r="934">
+      <c r="C934" s="10"/>
+    </row>
+    <row r="935">
+      <c r="C935" s="10"/>
+    </row>
+    <row r="936">
+      <c r="C936" s="10"/>
+    </row>
+    <row r="937">
+      <c r="C937" s="10"/>
+    </row>
+    <row r="938">
+      <c r="C938" s="10"/>
+    </row>
+    <row r="939">
+      <c r="C939" s="10"/>
+    </row>
+    <row r="940">
+      <c r="C940" s="10"/>
+    </row>
+    <row r="941">
+      <c r="C941" s="10"/>
+    </row>
+    <row r="942">
+      <c r="C942" s="10"/>
+    </row>
+    <row r="943">
+      <c r="C943" s="10"/>
+    </row>
+    <row r="944">
+      <c r="C944" s="10"/>
+    </row>
+    <row r="945">
+      <c r="C945" s="10"/>
+    </row>
+    <row r="946">
+      <c r="C946" s="10"/>
+    </row>
+    <row r="947">
+      <c r="C947" s="10"/>
+    </row>
+    <row r="948">
+      <c r="C948" s="10"/>
+    </row>
+    <row r="949">
+      <c r="C949" s="10"/>
+    </row>
+    <row r="950">
+      <c r="C950" s="10"/>
+    </row>
+    <row r="951">
+      <c r="C951" s="10"/>
+    </row>
+    <row r="952">
+      <c r="C952" s="10"/>
+    </row>
+    <row r="953">
+      <c r="C953" s="10"/>
+    </row>
+    <row r="954">
+      <c r="C954" s="10"/>
+    </row>
+    <row r="955">
+      <c r="C955" s="10"/>
+    </row>
+    <row r="956">
+      <c r="C956" s="10"/>
+    </row>
+    <row r="957">
+      <c r="C957" s="10"/>
+    </row>
+    <row r="958">
+      <c r="C958" s="10"/>
+    </row>
+    <row r="959">
+      <c r="C959" s="10"/>
+    </row>
+    <row r="960">
+      <c r="C960" s="10"/>
+    </row>
+    <row r="961">
+      <c r="C961" s="10"/>
+    </row>
+    <row r="962">
+      <c r="C962" s="10"/>
+    </row>
+    <row r="963">
+      <c r="C963" s="10"/>
+    </row>
+    <row r="964">
+      <c r="C964" s="10"/>
+    </row>
+    <row r="965">
+      <c r="C965" s="10"/>
+    </row>
+    <row r="966">
+      <c r="C966" s="10"/>
+    </row>
+    <row r="967">
+      <c r="C967" s="10"/>
+    </row>
+    <row r="968">
+      <c r="C968" s="10"/>
+    </row>
+    <row r="969">
+      <c r="C969" s="10"/>
+    </row>
+    <row r="970">
+      <c r="C970" s="10"/>
+    </row>
+    <row r="971">
+      <c r="C971" s="10"/>
+    </row>
+    <row r="972">
+      <c r="C972" s="10"/>
+    </row>
+    <row r="973">
+      <c r="C973" s="10"/>
+    </row>
+    <row r="974">
+      <c r="C974" s="10"/>
+    </row>
+    <row r="975">
+      <c r="C975" s="10"/>
+    </row>
+    <row r="976">
+      <c r="C976" s="10"/>
+    </row>
+    <row r="977">
+      <c r="C977" s="10"/>
+    </row>
+    <row r="978">
+      <c r="C978" s="10"/>
+    </row>
+    <row r="979">
+      <c r="C979" s="10"/>
+    </row>
+    <row r="980">
+      <c r="C980" s="10"/>
+    </row>
+    <row r="981">
+      <c r="C981" s="10"/>
+    </row>
+    <row r="982">
+      <c r="C982" s="10"/>
+    </row>
+    <row r="983">
+      <c r="C983" s="10"/>
+    </row>
+    <row r="984">
+      <c r="C984" s="10"/>
+    </row>
+    <row r="985">
+      <c r="C985" s="10"/>
+    </row>
+    <row r="986">
+      <c r="C986" s="10"/>
+    </row>
+    <row r="987">
+      <c r="C987" s="10"/>
+    </row>
+    <row r="988">
+      <c r="C988" s="10"/>
+    </row>
+    <row r="989">
+      <c r="C989" s="10"/>
+    </row>
+    <row r="990">
+      <c r="C990" s="10"/>
+    </row>
+    <row r="991">
+      <c r="C991" s="10"/>
+    </row>
+    <row r="992">
+      <c r="C992" s="10"/>
+    </row>
+    <row r="993">
+      <c r="C993" s="10"/>
+    </row>
+    <row r="994">
+      <c r="C994" s="10"/>
+    </row>
+    <row r="995">
+      <c r="C995" s="10"/>
+    </row>
+    <row r="996">
+      <c r="C996" s="10"/>
+    </row>
+    <row r="997">
+      <c r="C997" s="10"/>
+    </row>
+    <row r="998">
+      <c r="C998" s="10"/>
+    </row>
+    <row r="999">
+      <c r="C999" s="10"/>
+    </row>
+    <row r="1000">
+      <c r="C1000" s="10"/>
+    </row>
+  </sheetData>
+  <drawing r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>